<commit_message>
import data excel file updates for landscape data (lucc+biogeo)
</commit_message>
<xml_diff>
--- a/lucas/import_data/utility/observation/excel/apparatus.xlsx
+++ b/lucas/import_data/utility/observation/excel/apparatus.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="73">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -218,6 +218,27 @@
   </si>
   <si>
     <t xml:space="preserve">A wet sieving apparatus is a specialized laboratory device used to measure the aggregate stability of soil.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">human interpreter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">human sensing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human interpretation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human interpretation of usually nominal conditions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compilation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compilation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compilation of 2 or more data sources to a single dataset.</t>
   </si>
 </sst>
 </file>
@@ -227,7 +248,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -248,6 +269,11 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -292,7 +318,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -302,6 +328,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -325,37 +355,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -428,8 +458,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.74"/>
@@ -686,6 +716,34 @@
       </c>
       <c r="D18" s="1" t="s">
         <v>65</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>